<commit_message>
Sweep 14/08: add 4 new potential deals
Potential Deals (EARLY STAGE / NEGOTIATING):
- Quadrant Shopping Centre, Dunstable (Fast Forward Capital) - indic. terms £6.816m, 80% LTV, 12%, 12mo
- Lindsey House, 57-60 Lincoln's Inn Fields WC2 (City Financial Mortgages) - TS issued £10.8m, 11%, 9mo
- London Retail Parade Portfolio, 5 parades (Mantra/Prideview) - indic. £5.6m, 70% LTV, 11%, 18mo
- Flats 1 & 2 De Vere Gardens, Kensington W8 (IPCA) - enquiry, terms TBC

Skipped ongoing/existing: DNA Uxbridge extension, Elysian Stanmore, LandlordInvest JV paper.
State: bump last_sweep_utc to 2026-08-14; log conversations handled.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbSriq6UGNWFocVGvEFtNh
</commit_message>
<xml_diff>
--- a/Deals_Sheet_REL.xlsx
+++ b/Deals_Sheet_REL.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1164" uniqueCount="374">
   <si>
     <t xml:space="preserve">REL Finance Deals Sheet </t>
   </si>
@@ -277,6 +277,45 @@
     <t xml:space="preserve">DA received 17/07 via GLPG (Nick Swerner) / OakNorth (Hemesh Patel). 360-studio PBSA, GDV £148.6m, LTC 81%, LTGDV 61%, site PP £18.5m, 30-month term. Well above usual REL ticket — role for REL TBC (review).</t>
   </si>
   <si>
+    <t xml:space="preserve">Quadrant Shopping Centre, Dunstable, LU5 4RH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MGI Dunstable Ltd (Malhotra/Jain)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicative terms 12/08 via Darshan Daswani (Fast Forward Capital): £6.816m at 80% LTV/LTPP, 12% p.a., 1% arr fee, 1.5% exit, 12mo, PGs 20%. Acquisition of freehold shopping-centre parade (owner MGI Dunstable Ltd), rent ~£1.18m gross. Borrower countering 15mo term / nil exit / 12%; REL countered 1.5% arr + 12.75% if exit removed. Competing quotes (Shawbrook, WestOne). No formal TS yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lindsey House, 57-60 Lincoln's Inn Fields, WC2A 3LJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lindsey 21 Ltd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TS issued 12/08 via Manish Babla (City Financial Mortgages). Acquisition of Lindsey House, 57-60 Lincolns Inn Fields WC2. £10.8m gross / £9.72m net, 11% fixed, 9mo, 1.75% arr fee (incl 0.75% debt advisory), £243k exit, £891k interest reserve; guarantee capped £2.7m. Sized on lower of 65% MV (£16.615m) / 80% PP (£13.5m). Red Book val received 11/08. Planning/change-of-use angle. Offer valid to 26/08.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">London Retail Parade Portfolio (5 parades, 29 units - Woodford/E17/SE13/SE12/Bexley)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eastway Estates Ltd (Prideview Group)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicative terms 05/08 via Rickesh Patel (Mantra Commercial). Acquisition of 5 mixed-use retail parades (29 units) by Prideview SPV Eastway Estates Ltd. £5.6m at lower of 70% LTV (block value £8.0m) / 85.5% LTPP (PP £6.55m), 11% p.a., 1% arr, 1.5% exit, 18mo, PG 20%. Borrower requesting 24mo term / +6mo extension option. Value-add then refi/sell exit. No formal TS yet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flats 1 &amp; 2, De Vere Gardens, Kensington, W8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ladi (via IPCA Group)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enquiry 07/08 via Jignesh Desai (IPCA Group). Acquisition of combined Flats 1&amp;2, De Vere Gardens, Kensington W8 by "Ladi" from receivers at £4.5m (was £7m 2yrs ago); expected rent ~£4,300pw. Targeting end-Aug drawdown. REL indicated 60-70% LTV, 9.0-10.8% p.a., 1% arr, 1% exit, 12mo - awaiting pack, loan amount TBC, no formal terms issued.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dead Deals</t>
   </si>
   <si>
@@ -309,9 +348,6 @@
   </si>
   <si>
     <t xml:space="preserve">Burlington Gate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resi</t>
   </si>
   <si>
     <t xml:space="preserve">HNW</t>
@@ -1310,10 +1346,7 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="98">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -1340,7 +1373,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="19" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1396,7 +1429,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1420,7 +1453,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1452,7 +1485,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1492,7 +1525,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="2" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1536,7 +1569,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1544,11 +1577,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1564,7 +1597,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1572,23 +1605,23 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1612,7 +1645,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="2" borderId="0" xfId="19" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1624,7 +1657,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1648,7 +1681,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1672,7 +1705,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="7" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1680,7 +1713,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1696,7 +1729,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="19" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1961,7 +1994,7 @@
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:W41"/>
+  <dimension ref="A1:W45"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.29"/>
@@ -2175,7 +2208,7 @@
       <c r="U7" s="10"/>
       <c r="V7" s="10"/>
     </row>
-    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11"/>
       <c r="B8" s="11"/>
       <c r="C8" s="22"/>
@@ -2195,7 +2228,7 @@
       <c r="Q8" s="11"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11"/>
       <c r="B9" s="11"/>
       <c r="C9" s="22"/>
@@ -2215,7 +2248,7 @@
       <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
     </row>
-    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11"/>
       <c r="B10" s="11"/>
       <c r="C10" s="22"/>
@@ -2235,7 +2268,7 @@
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
     </row>
-    <row r="11" s="36" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" s="36" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
         <v>20</v>
       </c>
@@ -2273,7 +2306,7 @@
       <c r="U11" s="10"/>
       <c r="V11" s="10"/>
     </row>
-    <row r="12" s="36" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="36" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="37"/>
       <c r="B12" s="38"/>
       <c r="C12" s="39"/>
@@ -2297,7 +2330,7 @@
       <c r="U12" s="10"/>
       <c r="V12" s="10"/>
     </row>
-    <row r="13" customFormat="false" ht="12.75" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="12.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11"/>
       <c r="B13" s="38"/>
       <c r="C13" s="39"/>
@@ -2321,7 +2354,7 @@
       <c r="U13" s="10"/>
       <c r="V13" s="10"/>
     </row>
-    <row r="14" s="36" customFormat="true" ht="12.75" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" s="36" customFormat="true" ht="12.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
       <c r="B14" s="38"/>
       <c r="C14" s="39"/>
@@ -2345,7 +2378,7 @@
       <c r="U14" s="10"/>
       <c r="V14" s="10"/>
     </row>
-    <row r="15" s="36" customFormat="true" ht="12.75" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" s="36" customFormat="true" ht="12.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="37"/>
       <c r="B15" s="38"/>
       <c r="C15" s="39"/>
@@ -2369,7 +2402,7 @@
       <c r="U15" s="10"/>
       <c r="V15" s="10"/>
     </row>
-    <row r="16" s="36" customFormat="true" ht="12.75" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" s="36" customFormat="true" ht="12.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="37"/>
       <c r="B16" s="45" t="s">
         <v>3</v>
@@ -2399,7 +2432,7 @@
       <c r="U16" s="10"/>
       <c r="V16" s="10"/>
     </row>
-    <row r="17" customFormat="false" ht="12.75" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="12.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11"/>
       <c r="B17" s="38"/>
       <c r="C17" s="39"/>
@@ -2509,7 +2542,7 @@
       <c r="U19" s="10"/>
       <c r="V19" s="10"/>
     </row>
-    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="56" t="n">
         <v>46054</v>
       </c>
@@ -2566,7 +2599,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="56" t="n">
         <v>46082</v>
       </c>
@@ -2679,7 +2712,7 @@
       <c r="U22" s="10"/>
       <c r="V22" s="10"/>
     </row>
-    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="56" t="n">
         <v>46143</v>
       </c>
@@ -2735,7 +2768,7 @@
       <c r="U23" s="10"/>
       <c r="V23" s="10"/>
     </row>
-    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="56" t="n">
         <v>46143</v>
       </c>
@@ -2791,7 +2824,7 @@
       <c r="U24" s="10"/>
       <c r="V24" s="10"/>
     </row>
-    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="56" t="n">
         <v>46143</v>
       </c>
@@ -2847,7 +2880,7 @@
       <c r="U25" s="10"/>
       <c r="V25" s="10"/>
     </row>
-    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="56" t="n">
         <v>46174</v>
       </c>
@@ -2903,7 +2936,7 @@
       <c r="U26" s="10"/>
       <c r="V26" s="10"/>
     </row>
-    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="56" t="n">
         <v>46174</v>
       </c>
@@ -2960,7 +2993,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="56" t="n">
         <v>46174</v>
       </c>
@@ -3012,7 +3045,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="56" t="n">
         <v>46174</v>
       </c>
@@ -3064,7 +3097,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="56" t="n">
         <v>46204</v>
       </c>
@@ -3116,7 +3149,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="56" t="n">
         <v>46204</v>
       </c>
@@ -3160,7 +3193,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="56" t="n">
         <v>46204</v>
       </c>
@@ -3217,7 +3250,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="56" t="n">
         <v>46204</v>
       </c>
@@ -3270,103 +3303,320 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="56"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="23"/>
-      <c r="K34" s="23"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="22"/>
-      <c r="N34" s="26"/>
-      <c r="O34" s="27"/>
-      <c r="P34" s="22"/>
-      <c r="Q34" s="11"/>
-      <c r="R34" s="11"/>
-    </row>
-    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="28" t="s">
+    <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="56" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F34" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="H34" s="23" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J34" s="23" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="K34" s="23" t="n">
+        <v>8.52</v>
+      </c>
+      <c r="L34" s="25" t="n">
+        <f aca="false">J34/K34</f>
+        <v>0.800469483568075</v>
+      </c>
+      <c r="M34" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="N34" s="26" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="O34" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="P34" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q34" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="R34" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="56" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E35" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F35" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="G35" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="H35" s="23" t="n">
+        <v>9.72</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J35" s="23" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="K35" s="23" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="L35" s="25" t="n">
+        <f aca="false">J35/K35</f>
+        <v>0.649819494584838</v>
+      </c>
+      <c r="M35" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="N35" s="26" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="O35" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="P35" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q35" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="R35" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="56" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E36" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F36" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="G36" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="H36" s="23" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="I36" s="24" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J36" s="23" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K36" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="L36" s="25" t="n">
+        <f aca="false">J36/K36</f>
+        <v>0.7</v>
+      </c>
+      <c r="M36" s="22" t="n">
+        <v>18</v>
+      </c>
+      <c r="N36" s="26" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="O36" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="P36" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q36" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="R36" s="11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="56" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="D37" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="F37" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="H37" s="23"/>
+      <c r="I37" s="24"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="L37" s="25"/>
+      <c r="M37" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="N37" s="26"/>
+      <c r="O37" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="P37" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q37" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="R37" s="11" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="56"/>
+      <c r="B38" s="11"/>
+      <c r="C38" s="22"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="22"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="24"/>
+      <c r="J38" s="23"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="25"/>
+      <c r="M38" s="22"/>
+      <c r="N38" s="26"/>
+      <c r="O38" s="27"/>
+      <c r="P38" s="22"/>
+      <c r="Q38" s="11"/>
+      <c r="R38" s="11"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="60"/>
-      <c r="D35" s="61"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="60"/>
-      <c r="H35" s="31" t="n">
-        <f aca="false">SUM(H20:H34)</f>
-        <v>182.67</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <f aca="false">SUM(I20:I34)</f>
-        <v>2.313</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <f aca="false">SUM(J20:J34)</f>
-        <v>186.44</v>
-      </c>
-      <c r="K35" s="31" t="n">
-        <f aca="false">SUM(K20:K34)</f>
-        <v>336.44</v>
-      </c>
-      <c r="L35" s="32" t="n">
-        <f aca="false">AVERAGE(L20:L34)</f>
-        <v>0.607303103326683</v>
-      </c>
-      <c r="M35" s="60"/>
-      <c r="N35" s="62"/>
-      <c r="O35" s="60"/>
-      <c r="P35" s="60"/>
-      <c r="Q35" s="61"/>
-      <c r="R35" s="61"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="U39" s="1" t="n">
+      <c r="B39" s="28"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="61"/>
+      <c r="E39" s="60"/>
+      <c r="F39" s="11"/>
+      <c r="G39" s="60"/>
+      <c r="H39" s="31" t="n">
+        <f aca="false">SUM(H20:H37)</f>
+        <v>204.68</v>
+      </c>
+      <c r="I39" s="31" t="n">
+        <f aca="false">SUM(I20:I37)</f>
+        <v>5.683</v>
+      </c>
+      <c r="J39" s="31" t="n">
+        <f aca="false">SUM(J20:J37)</f>
+        <v>209.66</v>
+      </c>
+      <c r="K39" s="31" t="n">
+        <f aca="false">SUM(K20:K37)</f>
+        <v>374.08</v>
+      </c>
+      <c r="L39" s="32" t="n">
+        <f aca="false">AVERAGE(L20:L37)</f>
+        <v>0.627826832587487</v>
+      </c>
+      <c r="M39" s="60"/>
+      <c r="N39" s="62"/>
+      <c r="O39" s="60"/>
+      <c r="P39" s="60"/>
+      <c r="Q39" s="61"/>
+      <c r="R39" s="61"/>
+    </row>
+    <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U43" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="V39" s="63" t="n">
+      <c r="V43" s="63" t="n">
         <v>0.14</v>
       </c>
-      <c r="W39" s="1" t="n">
+      <c r="W43" s="1" t="n">
         <f aca="false">U36*V36</f>
         <v>0</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="64"/>
-      <c r="C40" s="65"/>
-      <c r="D40" s="65"/>
-      <c r="E40" s="66"/>
-      <c r="F40" s="65"/>
-      <c r="G40" s="67"/>
-      <c r="U40" s="1" t="n">
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="64"/>
+      <c r="C44" s="65"/>
+      <c r="D44" s="65"/>
+      <c r="E44" s="66"/>
+      <c r="F44" s="65"/>
+      <c r="G44" s="67"/>
+      <c r="U44" s="1" t="n">
         <v>0.9</v>
       </c>
-      <c r="V40" s="63" t="n">
+      <c r="V44" s="63" t="n">
         <v>0.02</v>
       </c>
-      <c r="W40" s="1" t="n">
+      <c r="W44" s="1" t="n">
         <f aca="false">U37*V37</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="64"/>
-      <c r="C41" s="65"/>
-      <c r="D41" s="65"/>
-      <c r="E41" s="66"/>
-      <c r="F41" s="65"/>
-      <c r="G41" s="67"/>
-      <c r="W41" s="1" t="n">
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="64"/>
+      <c r="C45" s="65"/>
+      <c r="D45" s="65"/>
+      <c r="E45" s="66"/>
+      <c r="F45" s="65"/>
+      <c r="G45" s="67"/>
+      <c r="W45" s="1" t="n">
         <f aca="false">W36+W37</f>
         <v>0</v>
       </c>
@@ -3394,7 +3644,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A3:V96"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="68" width="19.57"/>
@@ -3405,7 +3655,7 @@
   <sheetData>
     <row r="3" s="1" customFormat="true" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="69" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="C3" s="69"/>
       <c r="D3" s="46"/>
@@ -3435,7 +3685,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="E4" s="16" t="s">
         <v>6</v>
@@ -3445,16 +3695,16 @@
       </c>
       <c r="G4" s="16"/>
       <c r="H4" s="17" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="L4" s="19" t="s">
         <v>13</v>
@@ -3480,13 +3730,13 @@
     </row>
     <row r="5" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="C5" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>25</v>
@@ -3520,28 +3770,28 @@
         <v>0.103</v>
       </c>
       <c r="O5" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P5" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q5" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11"/>
       <c r="B6" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="30" t="s">
-        <v>93</v>
-      </c>
       <c r="D6" s="11" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>25</v>
@@ -3575,27 +3825,27 @@
         <v>0.12</v>
       </c>
       <c r="O6" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P6" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q6" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R6" s="75" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="11" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="C7" s="30" t="s">
         <v>32</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>25</v>
@@ -3629,28 +3879,28 @@
         <v>0.13</v>
       </c>
       <c r="O7" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P7" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q7" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R7" s="75" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11"/>
       <c r="B8" s="11" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C8" s="30" t="s">
         <v>32</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>25</v>
@@ -3684,28 +3934,28 @@
         <v>0.1</v>
       </c>
       <c r="O8" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P8" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q8" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R8" s="75" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="9" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="28"/>
       <c r="B9" s="11" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>66</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>25</v>
@@ -3739,28 +3989,28 @@
         <v>0.13</v>
       </c>
       <c r="O9" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P9" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q9" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R9" s="11" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="37"/>
       <c r="B10" s="11" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>32</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E10" s="22" t="s">
         <v>25</v>
@@ -3794,28 +4044,28 @@
         <v>0.1445</v>
       </c>
       <c r="O10" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P10" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q10" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R10" s="11" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="E11" s="22" t="s">
         <v>25</v>
@@ -3849,28 +4099,28 @@
         <v>0.13</v>
       </c>
       <c r="O11" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P11" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q11" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="37"/>
       <c r="B12" s="11" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C12" s="58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="E12" s="22" t="s">
         <v>25</v>
@@ -3904,28 +4154,28 @@
         <v>0.1435</v>
       </c>
       <c r="O12" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="P12" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q12" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R12" s="11" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="13" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="37"/>
       <c r="B13" s="11" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="C13" s="58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="E13" s="22" t="s">
         <v>25</v>
@@ -3959,28 +4209,28 @@
         <v>0.153</v>
       </c>
       <c r="O13" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="P13" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q13" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R13" s="11" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="37"/>
       <c r="B14" s="11" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="C14" s="58" t="s">
         <v>32</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E14" s="22" t="s">
         <v>25</v>
@@ -4014,28 +4264,28 @@
         <v>0.127</v>
       </c>
       <c r="O14" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="P14" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q14" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R14" s="11" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11"/>
       <c r="B15" s="11" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="E15" s="22" t="s">
         <v>25</v>
@@ -4069,28 +4319,28 @@
         <v>0.15</v>
       </c>
       <c r="O15" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P15" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q15" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R15" s="11" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="22"/>
       <c r="B16" s="11" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="C16" s="58" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="E16" s="22" t="s">
         <v>25</v>
@@ -4124,28 +4374,28 @@
         <v>0.131</v>
       </c>
       <c r="O16" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="P16" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q16" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R16" s="11" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11"/>
       <c r="B17" s="11" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="C17" s="58" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="E17" s="22" t="s">
         <v>25</v>
@@ -4179,28 +4429,28 @@
         <v>0.13</v>
       </c>
       <c r="O17" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P17" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q17" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R17" s="11" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11"/>
       <c r="B18" s="11" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="C18" s="58" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="E18" s="22" t="s">
         <v>25</v>
@@ -4234,28 +4484,28 @@
         <v>0.135</v>
       </c>
       <c r="O18" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P18" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q18" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R18" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="19" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="19" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11"/>
       <c r="B19" s="11" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="C19" s="58" t="s">
         <v>66</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="E19" s="22" t="s">
         <v>25</v>
@@ -4289,28 +4539,28 @@
         <v>0.139</v>
       </c>
       <c r="O19" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P19" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q19" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R19" s="11" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11"/>
       <c r="B20" s="11" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C20" s="58" t="s">
         <v>32</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="E20" s="22" t="s">
         <v>25</v>
@@ -4344,31 +4594,31 @@
         <v>0.147</v>
       </c>
       <c r="O20" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P20" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q20" s="11" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="R20" s="11" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11"/>
       <c r="B21" s="11" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C21" s="58" t="s">
         <v>32</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F21" s="22" t="s">
         <v>26</v>
@@ -4398,20 +4648,20 @@
         <v>0.215</v>
       </c>
       <c r="O21" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P21" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q21" s="11" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="R21" s="11"/>
     </row>
     <row r="22" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11"/>
       <c r="B22" s="11" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C22" s="58" t="s">
         <v>32</v>
@@ -4434,10 +4684,10 @@
     </row>
     <row r="23" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="11" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="22" t="s">
@@ -4472,37 +4722,37 @@
         <v>0.165</v>
       </c>
       <c r="O23" s="22" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="P23" s="22" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="Q23" s="11" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="R23" s="11" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11"/>
       <c r="B24" s="76" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="C24" s="77" t="s">
         <v>32</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="E24" s="78" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F24" s="78" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="78" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="H24" s="79" t="n">
         <v>4.33</v>
@@ -4526,34 +4776,34 @@
         <v>0.24</v>
       </c>
       <c r="O24" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P24" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q24" s="11" t="s">
         <v>75</v>
       </c>
       <c r="R24" s="11" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
     </row>
     <row r="25" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11"/>
       <c r="B25" s="11" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="C25" s="58" t="s">
         <v>32</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="G25" s="22" t="s">
         <v>51</v>
@@ -4581,28 +4831,28 @@
         <v>0.153</v>
       </c>
       <c r="O25" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P25" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q25" s="11" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="R25" s="11" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="26" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="26" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11"/>
       <c r="B26" s="11" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>32</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="E26" s="22" t="s">
         <v>25</v>
@@ -4635,29 +4885,29 @@
         <v>0.152</v>
       </c>
       <c r="O26" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P26" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q26" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R26" s="11"/>
     </row>
-    <row r="27" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11"/>
       <c r="B27" s="11" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="F27" s="22" t="s">
         <v>26</v>
@@ -4687,26 +4937,26 @@
         <v>0.15</v>
       </c>
       <c r="O27" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="P27" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q27" s="11" t="s">
         <v>29</v>
       </c>
       <c r="R27" s="11"/>
     </row>
-    <row r="28" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11"/>
       <c r="B28" s="11" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>32</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="E28" s="22" t="s">
         <v>25</v>
@@ -4740,10 +4990,10 @@
         <v>0.1288</v>
       </c>
       <c r="O28" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P28" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q28" s="11" t="s">
         <v>75</v>
@@ -4753,7 +5003,7 @@
     <row r="29" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11"/>
       <c r="B29" s="11" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>32</v>
@@ -4791,10 +5041,10 @@
         <v>0.1394</v>
       </c>
       <c r="O29" s="27" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="P29" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q29" s="11" t="s">
         <v>29</v>
@@ -4804,18 +5054,18 @@
       <c r="T29" s="10"/>
       <c r="U29" s="10"/>
     </row>
-    <row r="30" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="56" t="n">
         <v>45689</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="E30" s="22" t="s">
         <v>25</v>
@@ -4859,18 +5109,18 @@
       </c>
       <c r="R30" s="11"/>
     </row>
-    <row r="31" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="56" t="n">
         <v>45717</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="E31" s="22" t="s">
         <v>25</v>
@@ -4914,21 +5164,21 @@
       </c>
       <c r="R31" s="11"/>
       <c r="S31" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="32" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="32" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="56" t="n">
         <v>45717</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="E32" s="22" t="s">
         <v>25</v>
@@ -4972,21 +5222,21 @@
       </c>
       <c r="R32" s="11"/>
       <c r="S32" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="33" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="33" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="56" t="n">
         <v>45717</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="E33" s="22" t="s">
         <v>25</v>
@@ -5028,21 +5278,21 @@
       </c>
       <c r="R33" s="11"/>
       <c r="S33" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="34" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="34" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="56" t="n">
         <v>45689</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="C34" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="E34" s="22" t="s">
         <v>25</v>
@@ -5085,27 +5335,27 @@
         <v>29</v>
       </c>
       <c r="R34" s="11" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="S34" s="1" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="35" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="35" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="56" t="n">
         <v>45717</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="C35" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F35" s="22" t="s">
         <v>26</v>
@@ -5144,24 +5394,24 @@
         <v>75</v>
       </c>
       <c r="R35" s="11" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="S35" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="36" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="36" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="E36" s="22" t="s">
         <v>25</v>
@@ -5205,21 +5455,21 @@
       </c>
       <c r="R36" s="11"/>
       <c r="S36" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="37" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="37" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="E37" s="22" t="s">
         <v>25</v>
@@ -5263,21 +5513,21 @@
       </c>
       <c r="R37" s="11"/>
       <c r="S37" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="38" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="38" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="C38" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="E38" s="22" t="s">
         <v>25</v>
@@ -5322,18 +5572,18 @@
       </c>
       <c r="R38" s="11"/>
     </row>
-    <row r="39" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="C39" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E39" s="22" t="s">
         <v>25</v>
@@ -5377,21 +5627,21 @@
       </c>
       <c r="R39" s="11"/>
       <c r="S39" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="40" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="40" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="C40" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E40" s="22" t="s">
         <v>25</v>
@@ -5435,21 +5685,21 @@
       </c>
       <c r="R40" s="11"/>
       <c r="S40" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="41" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="41" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="56" t="n">
         <v>45772</v>
       </c>
       <c r="B41" s="57" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="C41" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="E41" s="22" t="s">
         <v>25</v>
@@ -5493,7 +5743,7 @@
       </c>
       <c r="R41" s="11"/>
       <c r="S41" s="1" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
     </row>
     <row r="42" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5501,13 +5751,13 @@
         <v>45778</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="E42" s="22" t="s">
         <v>25</v>
@@ -5550,21 +5800,21 @@
         <v>29</v>
       </c>
       <c r="R42" s="11" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="43" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="43" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="E43" s="22" t="s">
         <v>25</v>
@@ -5607,24 +5857,24 @@
         <v>29</v>
       </c>
       <c r="R43" s="11" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="S43" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="44" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="44" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="E44" s="22" t="s">
         <v>25</v>
@@ -5667,24 +5917,24 @@
         <v>29</v>
       </c>
       <c r="R44" s="11" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="S44" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="45" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="45" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="56" t="n">
         <v>45748</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="C45" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="E45" s="22" t="s">
         <v>25</v>
@@ -5727,10 +5977,10 @@
         <v>75</v>
       </c>
       <c r="R45" s="11" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="S45" s="1" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
     </row>
     <row r="46" s="1" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5738,13 +5988,13 @@
         <v>45772</v>
       </c>
       <c r="B46" s="81" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="E46" s="22" t="s">
         <v>25</v>
@@ -5788,18 +6038,18 @@
       </c>
       <c r="R46" s="11"/>
     </row>
-    <row r="47" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="56" t="n">
         <v>45778</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="C47" s="22" t="s">
         <v>66</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E47" s="22" t="s">
         <v>25</v>
@@ -5843,18 +6093,18 @@
       </c>
       <c r="R47" s="11"/>
     </row>
-    <row r="48" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="56" t="n">
         <v>45809</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="E48" s="22" t="s">
         <v>25</v>
@@ -5894,21 +6144,21 @@
       </c>
       <c r="R48" s="11"/>
       <c r="S48" s="1" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="49" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="49" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="56" t="n">
         <v>45809</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="E49" s="22" t="s">
         <v>25</v>
@@ -5948,24 +6198,24 @@
         <v>28</v>
       </c>
       <c r="Q49" s="11" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="R49" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="50" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="50" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="56" t="n">
         <v>45809</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="C50" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D50" s="11" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="E50" s="22" t="s">
         <v>25</v>
@@ -6008,7 +6258,7 @@
         <v>29</v>
       </c>
       <c r="R50" s="11" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6016,13 +6266,13 @@
         <v>45901</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="C51" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="E51" s="22" t="s">
         <v>25</v>
@@ -6061,27 +6311,27 @@
         <v>29</v>
       </c>
       <c r="R51" s="11" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="S51" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="52" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="52" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="82" t="n">
         <v>45901</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F52" s="22" t="s">
         <v>26</v>
@@ -6121,24 +6371,24 @@
         <v>29</v>
       </c>
       <c r="R52" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="53" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="53" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="82" t="n">
         <v>45901</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="C53" s="22" t="s">
         <v>66</v>
       </c>
       <c r="D53" s="11" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F53" s="22" t="s">
         <v>26</v>
@@ -6178,24 +6428,24 @@
         <v>29</v>
       </c>
       <c r="R53" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="54" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="54" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D54" s="11" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="F54" s="22" t="s">
         <v>26</v>
@@ -6235,21 +6485,21 @@
         <v>29</v>
       </c>
       <c r="R54" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="55" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="55" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="C55" s="22" t="s">
         <v>66</v>
       </c>
       <c r="D55" s="11" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="E55" s="22" t="s">
         <v>25</v>
@@ -6292,21 +6542,21 @@
         <v>29</v>
       </c>
       <c r="R55" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="56" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="56" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B56" s="58" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="E56" s="22" t="s">
         <v>25</v>
@@ -6349,21 +6599,21 @@
         <v>75</v>
       </c>
       <c r="R56" s="11" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="57" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="57" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B57" s="83" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="C57" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D57" s="85" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="E57" s="84" t="s">
         <v>25</v>
@@ -6406,21 +6656,21 @@
         <v>29</v>
       </c>
       <c r="R57" s="85" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="58" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="58" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B58" s="83" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="C58" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D58" s="85" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="E58" s="84" t="s">
         <v>25</v>
@@ -6449,22 +6699,22 @@
         <v>29</v>
       </c>
       <c r="R58" s="85" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="59" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B59" s="83" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="C59" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D59" s="85"/>
       <c r="E59" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F59" s="84" t="s">
         <v>26</v>
@@ -6504,24 +6754,24 @@
         <v>29</v>
       </c>
       <c r="R59" s="85" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="60" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="60" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B60" s="83" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="C60" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D60" s="85" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="E60" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F60" s="84" t="s">
         <v>26</v>
@@ -6561,15 +6811,15 @@
         <v>29</v>
       </c>
       <c r="R60" s="85" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="61" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="61" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B61" s="83" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="C61" s="84" t="s">
         <v>32</v>
@@ -6616,21 +6866,21 @@
         <v>29</v>
       </c>
       <c r="R61" s="85" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="S61" s="1" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="62" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="62" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="82" t="n">
         <v>46082</v>
       </c>
       <c r="B62" s="91" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="C62" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D62" s="83"/>
       <c r="E62" s="84" t="s">
@@ -6669,21 +6919,21 @@
       </c>
       <c r="R62" s="85"/>
     </row>
-    <row r="63" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="82" t="n">
         <v>46082</v>
       </c>
       <c r="B63" s="91" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="C63" s="84" t="s">
         <v>54</v>
       </c>
       <c r="D63" s="83" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="E63" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F63" s="84" t="s">
         <v>26</v>
@@ -6715,24 +6965,24 @@
       </c>
       <c r="Q63" s="85"/>
       <c r="R63" s="85" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="64" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="64" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="82" t="n">
         <v>46023</v>
       </c>
       <c r="B64" s="83" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="C64" s="84" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D64" s="85" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E64" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F64" s="84" t="s">
         <v>26</v>
@@ -6771,24 +7021,24 @@
         <v>29</v>
       </c>
       <c r="R64" s="85" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="S64" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="65" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="65" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B65" s="83" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="C65" s="84" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="D65" s="85" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="E65" s="84" t="s">
         <v>25</v>
@@ -6831,24 +7081,24 @@
         <v>29</v>
       </c>
       <c r="R65" s="85" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="S65" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="66" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="66" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="82" t="n">
         <v>46023</v>
       </c>
       <c r="B66" s="83" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="C66" s="84" t="s">
         <v>54</v>
       </c>
       <c r="D66" s="85" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="E66" s="84"/>
       <c r="F66" s="84" t="s">
@@ -6879,27 +7129,27 @@
         <v>29</v>
       </c>
       <c r="R66" s="85" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="S66" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="67" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="67" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="82" t="n">
         <v>45901</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="C67" s="22" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D67" s="58" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="E67" s="22" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F67" s="22" t="s">
         <v>26</v>
@@ -6939,27 +7189,27 @@
         <v>29</v>
       </c>
       <c r="R67" s="11" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="S67" s="1" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="68" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="68" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B68" s="58" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="C68" s="22" t="s">
         <v>66</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="E68" s="22" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="F68" s="22" t="s">
         <v>26</v>
@@ -6999,25 +7249,25 @@
         <v>29</v>
       </c>
       <c r="R68" s="11" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="S68" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="69" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="69" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B69" s="83" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="C69" s="84" t="s">
         <v>54</v>
       </c>
       <c r="D69" s="85"/>
       <c r="E69" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F69" s="84" t="s">
         <v>26</v>
@@ -7057,22 +7307,22 @@
         <v>29</v>
       </c>
       <c r="R69" s="85" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="70" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="70" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B70" s="83" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="C70" s="84" t="s">
         <v>32</v>
       </c>
       <c r="D70" s="85"/>
       <c r="E70" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F70" s="84" t="s">
         <v>26</v>
@@ -7089,7 +7339,7 @@
       </c>
       <c r="K70" s="86"/>
       <c r="L70" s="88" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="M70" s="84"/>
       <c r="N70" s="89"/>
@@ -7100,18 +7350,18 @@
       <c r="Q70" s="85"/>
       <c r="R70" s="85"/>
     </row>
-    <row r="71" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B71" s="83" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="C71" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D71" s="85" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="E71" s="84" t="s">
         <v>25</v>
@@ -7154,27 +7404,27 @@
         <v>29</v>
       </c>
       <c r="R71" s="85" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="S71" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="72" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="72" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B72" s="83" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="C72" s="84" t="s">
         <v>54</v>
       </c>
       <c r="D72" s="85" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="E72" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F72" s="84" t="s">
         <v>26</v>
@@ -7214,27 +7464,27 @@
         <v>29</v>
       </c>
       <c r="R72" s="85" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="S72" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="73" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="73" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="82" t="n">
         <v>45931</v>
       </c>
       <c r="B73" s="83" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="C73" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D73" s="85" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="E73" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F73" s="84" t="s">
         <v>26</v>
@@ -7260,21 +7510,21 @@
       <c r="Q73" s="85"/>
       <c r="R73" s="85"/>
     </row>
-    <row r="74" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="82" t="n">
         <v>46054</v>
       </c>
       <c r="B74" s="83" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="C74" s="84" t="s">
         <v>23</v>
       </c>
       <c r="D74" s="85" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="E74" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F74" s="84" t="s">
         <v>26</v>
@@ -7307,21 +7557,21 @@
       </c>
       <c r="R74" s="85"/>
     </row>
-    <row r="75" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="82" t="n">
         <v>46023</v>
       </c>
       <c r="B75" s="83" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="C75" s="84" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="D75" s="85" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="E75" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F75" s="84" t="s">
         <v>26</v>
@@ -7361,24 +7611,24 @@
         <v>29</v>
       </c>
       <c r="R75" s="85" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="76" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="76" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="82" t="n">
         <v>46054</v>
       </c>
       <c r="B76" s="57" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="C76" s="84" t="s">
         <v>66</v>
       </c>
       <c r="D76" s="83" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="E76" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F76" s="84" t="s">
         <v>26</v>
@@ -7418,24 +7668,24 @@
         <v>29</v>
       </c>
       <c r="R76" s="85" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="77" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="77" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="82" t="n">
         <v>46054</v>
       </c>
       <c r="B77" s="83" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="C77" s="84" t="s">
         <v>23</v>
       </c>
       <c r="D77" s="85" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="E77" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F77" s="84" t="s">
         <v>26</v>
@@ -7469,24 +7719,24 @@
         <v>29</v>
       </c>
       <c r="R77" s="85" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="78" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="78" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="82" t="n">
         <v>46054</v>
       </c>
       <c r="B78" s="91" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="C78" s="84" t="s">
         <v>23</v>
       </c>
       <c r="D78" s="83" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="E78" s="84" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="F78" s="84" t="s">
         <v>26</v>
@@ -7512,24 +7762,24 @@
       <c r="P78" s="84"/>
       <c r="Q78" s="85"/>
       <c r="R78" s="85" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="79" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="79" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="82" t="n">
         <v>46023</v>
       </c>
       <c r="B79" s="83" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="C79" s="84" t="s">
         <v>32</v>
       </c>
       <c r="D79" s="85" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="E79" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F79" s="84" t="s">
         <v>26</v>
@@ -7568,21 +7818,21 @@
         <v>29</v>
       </c>
       <c r="R79" s="85" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="80" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="80" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="82" t="n">
         <v>46023</v>
       </c>
       <c r="B80" s="83" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="C80" s="84" t="s">
         <v>66</v>
       </c>
       <c r="D80" s="85" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="E80" s="84" t="s">
         <v>25</v>
@@ -7624,24 +7874,24 @@
         <v>75</v>
       </c>
       <c r="R80" s="85" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="81" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="81" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="82" t="n">
         <v>46023</v>
       </c>
       <c r="B81" s="83" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="C81" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D81" s="85" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="E81" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F81" s="84" t="s">
         <v>26</v>
@@ -7680,21 +7930,21 @@
         <v>75</v>
       </c>
       <c r="R81" s="85" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="82" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="82" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="82" t="n">
         <v>46054</v>
       </c>
       <c r="B82" s="91" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="C82" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D82" s="83" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="E82" s="84" t="s">
         <v>25</v>
@@ -7737,24 +7987,24 @@
         <v>29</v>
       </c>
       <c r="R82" s="85" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="83" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="83" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="82" t="n">
         <v>46082</v>
       </c>
       <c r="B83" s="91" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="C83" s="84" t="s">
         <v>23</v>
       </c>
       <c r="D83" s="83" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="E83" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F83" s="84" t="s">
         <v>26</v>
@@ -7788,21 +8038,21 @@
       </c>
       <c r="Q83" s="85"/>
       <c r="R83" s="85" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="84" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="84" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="82" t="n">
         <v>46113</v>
       </c>
       <c r="B84" s="91" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="C84" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D84" s="83" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="E84" s="84" t="s">
         <v>25</v>
@@ -7840,22 +8090,22 @@
         <v>29</v>
       </c>
       <c r="R84" s="85" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="S84" s="92"/>
     </row>
-    <row r="85" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="82" t="n">
         <v>46113</v>
       </c>
       <c r="B85" s="91" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="C85" s="84" t="s">
         <v>23</v>
       </c>
       <c r="D85" s="83" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="E85" s="84" t="s">
         <v>25</v>
@@ -7895,22 +8145,22 @@
         <v>75</v>
       </c>
       <c r="R85" s="85" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="S85" s="92"/>
     </row>
-    <row r="86" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="82" t="n">
         <v>46143</v>
       </c>
       <c r="B86" s="91" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="C86" s="84" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="D86" s="83" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="E86" s="84" t="s">
         <v>25</v>
@@ -7948,13 +8198,13 @@
         <v>29</v>
       </c>
       <c r="R86" s="85" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="S86" s="92" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="87" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="87" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="82" t="n">
         <v>46143</v>
       </c>
@@ -8001,24 +8251,24 @@
         <v>29</v>
       </c>
       <c r="R87" s="85" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="S87" s="92" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="88" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="88" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="82" t="n">
         <v>46023</v>
       </c>
       <c r="B88" s="83" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="C88" s="84" t="s">
         <v>23</v>
       </c>
       <c r="D88" s="85" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="E88" s="84" t="s">
         <v>25</v>
@@ -8061,7 +8311,7 @@
         <v>29</v>
       </c>
       <c r="R88" s="85" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
     </row>
     <row r="89" s="1" customFormat="true" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8069,7 +8319,7 @@
         <v>46113</v>
       </c>
       <c r="B89" s="91" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C89" s="84" t="s">
         <v>23</v>
@@ -8111,25 +8361,25 @@
         <v>75</v>
       </c>
       <c r="R89" s="94" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="S89" s="59"/>
       <c r="T89" s="10"/>
       <c r="U89" s="10"/>
       <c r="V89" s="10"/>
     </row>
-    <row r="90" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="82" t="n">
         <v>46113</v>
       </c>
       <c r="B90" s="91" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="C90" s="84" t="s">
         <v>54</v>
       </c>
       <c r="D90" s="83" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="E90" s="84" t="s">
         <v>25</v>
@@ -8172,21 +8422,21 @@
       <c r="U90" s="10"/>
       <c r="V90" s="10"/>
     </row>
-    <row r="91" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="82" t="n">
         <v>46113</v>
       </c>
       <c r="B91" s="91" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C91" s="84" t="s">
         <v>32</v>
       </c>
       <c r="D91" s="83" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="E91" s="84" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="F91" s="84" t="s">
         <v>26</v>
@@ -8230,18 +8480,18 @@
       <c r="U91" s="10"/>
       <c r="V91" s="10"/>
     </row>
-    <row r="92" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="82" t="n">
         <v>46204</v>
       </c>
       <c r="B92" s="91" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="C92" s="84" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="D92" s="83" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="E92" s="84" t="s">
         <v>25</v>
@@ -8269,11 +8519,11 @@
         <v>75</v>
       </c>
       <c r="R92" s="85" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="S92" s="59"/>
     </row>
-    <row r="93" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="82"/>
       <c r="B93" s="91"/>
       <c r="C93" s="84"/>
@@ -8294,7 +8544,7 @@
       <c r="R93" s="85"/>
       <c r="S93" s="59"/>
     </row>
-    <row r="94" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="82"/>
       <c r="B94" s="91"/>
       <c r="C94" s="84"/>
@@ -8335,7 +8585,7 @@
       <c r="Q95" s="11"/>
       <c r="R95" s="11"/>
     </row>
-    <row r="96" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="28" t="s">
         <v>20</v>
       </c>
@@ -8392,7 +8642,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A3:X10"/>
-  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.70703125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="68" width="39.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="2" style="68" width="12.72"/>
@@ -8401,7 +8651,7 @@
   <sheetData>
     <row r="3" s="1" customFormat="true" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="69" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="B3" s="69"/>
       <c r="C3" s="49"/>
@@ -8434,10 +8684,10 @@
         <v>4</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="E4" s="16" t="s">
         <v>6</v>
@@ -8447,16 +8697,16 @@
       </c>
       <c r="G4" s="16"/>
       <c r="H4" s="17" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="L4" s="19" t="s">
         <v>13</v>
@@ -8468,10 +8718,10 @@
         <v>15</v>
       </c>
       <c r="O4" s="20" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="P4" s="20" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="Q4" s="16" t="s">
         <v>16</v>
@@ -8488,7 +8738,7 @@
     </row>
     <row r="5" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>32</v>
@@ -8497,7 +8747,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>25</v>
@@ -8530,25 +8780,25 @@
         <v>0.16</v>
       </c>
       <c r="O5" s="22" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="P5" s="22" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="Q5" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="R5" s="22" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="S5" s="11" t="s">
         <v>29</v>
       </c>
       <c r="T5" s="11" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="U5" s="96" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="V5" s="10"/>
       <c r="W5" s="10"/>
@@ -8556,7 +8806,7 @@
     </row>
     <row r="6" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="B6" s="58" t="s">
         <v>32</v>
@@ -8565,7 +8815,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>25</v>
@@ -8599,42 +8849,42 @@
         <v>0.133</v>
       </c>
       <c r="O6" s="26" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="P6" s="26" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="Q6" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="R6" s="22" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="S6" s="11" t="s">
         <v>29</v>
       </c>
       <c r="T6" s="11" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="U6" s="97" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="V6" s="10"/>
       <c r="W6" s="10"/>
       <c r="X6" s="10"/>
     </row>
-    <row r="7" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="56" t="n">
         <v>45778</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>25</v>
@@ -8668,39 +8918,39 @@
         <v>0.1458</v>
       </c>
       <c r="O7" s="27" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="P7" s="22" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="Q7" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="R7" s="11" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="S7" s="1" t="s">
         <v>29</v>
       </c>
       <c r="T7" s="11" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="8" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="56" t="n">
         <v>45809</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>25</v>
@@ -8734,25 +8984,25 @@
         <v>0.2511</v>
       </c>
       <c r="O8" s="27" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="P8" s="22" t="s">
         <v>28</v>
       </c>
       <c r="Q8" s="27" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="R8" s="11" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="S8" s="1" t="s">
         <v>75</v>
       </c>
       <c r="T8" s="11" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8780,7 +9030,7 @@
       <c r="W9" s="10"/>
       <c r="X9" s="10"/>
     </row>
-    <row r="10" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
Reorder Early-Stage deals by real date; condense comments
- Replace placeholder 1st-of-month dates with actual enquiry/TS dates on
  swept rows, so the section sorts chronologically (was interleaving Sep
  above Aug).
- Sort EARLY STAGE / NEGOTIATING block ascending by Date Received.
- Trim verbose Comments to one concise line per deal.
- Flag possible duplicate: new "Brighton Pier" (Sep) vs existing
  "Brighton Palace Pier" (Jun) - left both, noted for confirmation.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QbSriq6UGNWFocVGvEFtNh
</commit_message>
<xml_diff>
--- a/Deals_Sheet_REL.xlsx
+++ b/Deals_Sheet_REL.xlsx
@@ -2221,7 +2221,7 @@
       </c>
       <c r="R27" s="108" t="inlineStr">
         <is>
-          <t>Updated TS issued 14/07 at 62% LTV/LTPP (£6.82m day 1, 11.0% fixed, 1.25% fee) — TopCo guarantees/financials unavailable; rent charge + OpCo duty of care deed required. Awaiting countersigned TS and commitment fee.</t>
+          <t>Revised TS 14/07: 62% LTV, £6.82m, 11% fixed, 18m. Awaiting countersigned TS + fee. Broker Jignesh Desai (IPCA).</t>
         </is>
       </c>
     </row>
@@ -2443,21 +2443,21 @@
     </row>
     <row r="31" ht="12.75" customHeight="1" s="105">
       <c r="A31" s="155" t="n">
-        <v>46204</v>
+        <v>46212</v>
       </c>
       <c r="B31" s="108" t="inlineStr">
         <is>
-          <t>31-32 Rutland Gate &amp; 58-59 Montpelier Walk, SW7 1BN</t>
+          <t>Houndswood House Care Home, Harper Lane, Radlett WD7 7HU</t>
         </is>
       </c>
       <c r="C31" s="120" t="inlineStr">
         <is>
-          <t>Resi (Super Prime)</t>
+          <t>Care Home</t>
         </is>
       </c>
       <c r="D31" s="108" t="inlineStr">
         <is>
-          <t>Four Square (Saudi investor equity)</t>
+          <t>Anahi Properties Ltd (Hindocha)</t>
         </is>
       </c>
       <c r="E31" s="120" t="inlineStr">
@@ -2472,21 +2472,34 @@
       </c>
       <c r="G31" s="120" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H31" s="121" t="n"/>
-      <c r="I31" s="122" t="n"/>
-      <c r="J31" s="121" t="n"/>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H31" s="121" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="I31" s="122" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="J31" s="121" t="n">
+        <v>0.95</v>
+      </c>
       <c r="K31" s="121" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="L31" s="123" t="n"/>
-      <c r="M31" s="120" t="n"/>
-      <c r="N31" s="124" t="n"/>
+        <v>2.5</v>
+      </c>
+      <c r="L31" s="123">
+        <f>J32/K32</f>
+        <v/>
+      </c>
+      <c r="M31" s="120" t="n">
+        <v>12</v>
+      </c>
+      <c r="N31" s="124" t="n">
+        <v>0.1125</v>
+      </c>
       <c r="O31" s="125" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P31" s="120" t="inlineStr">
@@ -2496,32 +2509,32 @@
       </c>
       <c r="Q31" s="108" t="inlineStr">
         <is>
-          <t>Broker</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="R31" s="108" t="inlineStr">
         <is>
-          <t>Enquiry 14/07 via Lee Neenan (Irwell). Acquisition of 4 adjacent houses c.£18.5m + £9m refurb, GDV £37m. REL indicated up to 75% LTV/LTPP acquisition bridge (no dev finance). Detailed info list sent 15/07 — awaiting pack.</t>
+          <t>TS 09/07: £0.95m, 9.75%, 12m, 38% LTV. Anahi Properties. Offer lapsed 30/07 - chase.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="12.75" customHeight="1" s="105">
       <c r="A32" s="155" t="n">
-        <v>46204</v>
+        <v>46217</v>
       </c>
       <c r="B32" s="108" t="inlineStr">
         <is>
-          <t>Houndswood House Care Home, Harper Lane, Radlett WD7 7HU</t>
+          <t>31-32 Rutland Gate &amp; 58-59 Montpelier Walk, SW7 1BN</t>
         </is>
       </c>
       <c r="C32" s="120" t="inlineStr">
         <is>
-          <t>Care Home</t>
+          <t>Resi (Super Prime)</t>
         </is>
       </c>
       <c r="D32" s="108" t="inlineStr">
         <is>
-          <t>Anahi Properties Ltd (Hindocha)</t>
+          <t>Four Square (Saudi investor equity)</t>
         </is>
       </c>
       <c r="E32" s="120" t="inlineStr">
@@ -2536,34 +2549,21 @@
       </c>
       <c r="G32" s="120" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H32" s="121" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="I32" s="122" t="n">
-        <v>0.107</v>
-      </c>
-      <c r="J32" s="121" t="n">
-        <v>0.95</v>
-      </c>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H32" s="121" t="n"/>
+      <c r="I32" s="122" t="n"/>
+      <c r="J32" s="121" t="n"/>
       <c r="K32" s="121" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L32" s="123">
-        <f>J32/K32</f>
-        <v/>
-      </c>
-      <c r="M32" s="120" t="n">
-        <v>12</v>
-      </c>
-      <c r="N32" s="124" t="n">
-        <v>0.1125</v>
-      </c>
+        <v>18.5</v>
+      </c>
+      <c r="L32" s="123" t="n"/>
+      <c r="M32" s="120" t="n"/>
+      <c r="N32" s="124" t="n"/>
       <c r="O32" s="125" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P32" s="120" t="inlineStr">
@@ -2573,18 +2573,18 @@
       </c>
       <c r="Q32" s="108" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Broker</t>
         </is>
       </c>
       <c r="R32" s="108" t="inlineStr">
         <is>
-          <t>TS issued 09/07: 9.75% fixed, £92,625 interest reserve within facility, £9.5k arr fee + £4.75k exit fee, £280k joint PGs. Sized on 2024 KF VP value £2.5m / £3.5m 2024 purchase — no Red Book required. Refi of SBIUK £1.5m. Chased 16/07; offer valid to 30/07.</t>
+          <t>Enquiry 14/07; awaiting info pack. ~75% LTV acq bridge indicated. Irwell/Lee Neenan. Figures TBC.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="12.75" customHeight="1" s="105">
       <c r="A33" s="155" t="n">
-        <v>46204</v>
+        <v>46220</v>
       </c>
       <c r="B33" s="108" t="inlineStr">
         <is>
@@ -2651,27 +2651,27 @@
       </c>
       <c r="R33" s="108" t="inlineStr">
         <is>
-          <t>DA received 17/07 via GLPG (Nick Swerner) / OakNorth (Hemesh Patel). 360-studio PBSA, GDV £148.6m, LTC 81%, LTGDV 61%, site PP £18.5m, 30-month term. Well above usual REL ticket — role for REL TBC (review).</t>
+          <t>DA 17/07: £90.4m gross, GDV £148.6m, 30m PBSA. Via GLPG/OakNorth. REL role TBC.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="12.75" customHeight="1" s="105">
       <c r="A34" s="155" t="n">
-        <v>46235</v>
+        <v>46237</v>
       </c>
       <c r="B34" s="108" t="inlineStr">
         <is>
-          <t>Quadrant Shopping Centre, Dunstable, LU5 4RH</t>
+          <t>London Retail Parade Portfolio (5 parades, 29 units - Woodford/E17/SE13/SE12/Bexley)</t>
         </is>
       </c>
       <c r="C34" s="120" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Mixed-use</t>
         </is>
       </c>
       <c r="D34" s="108" t="inlineStr">
         <is>
-          <t>MGI Dunstable Ltd (Malhotra/Jain)</t>
+          <t>Eastway Estates Ltd (Prideview Group)</t>
         </is>
       </c>
       <c r="E34" s="120" t="inlineStr">
@@ -2690,26 +2690,26 @@
         </is>
       </c>
       <c r="H34" s="121" t="n">
-        <v>6.75</v>
+        <v>5.54</v>
       </c>
       <c r="I34" s="122" t="n">
-        <v>0.99</v>
+        <v>1.06</v>
       </c>
       <c r="J34" s="121" t="n">
-        <v>6.82</v>
+        <v>5.6</v>
       </c>
       <c r="K34" s="121" t="n">
-        <v>8.52</v>
+        <v>8</v>
       </c>
       <c r="L34" s="123">
-        <f>J34/K34</f>
+        <f>J36/K36</f>
         <v/>
       </c>
       <c r="M34" s="120" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N34" s="124" t="n">
-        <v>0.145</v>
+        <v>0.127</v>
       </c>
       <c r="O34" s="125" t="inlineStr">
         <is>
@@ -2728,13 +2728,13 @@
       </c>
       <c r="R34" s="108" t="inlineStr">
         <is>
-          <t>Indicative terms 12/08 via Darshan Daswani (Fast Forward Capital): £6.816m at 80% LTV/LTPP, 12% p.a., 1% arr fee, 1.5% exit, 12mo, PGs 20%. Acquisition of freehold shopping-centre parade (owner MGI Dunstable Ltd), rent ~£1.18m gross. Borrower countering 15mo term / nil exit / 12%; REL countered 1.5% arr + 12.75% if exit removed. Competing quotes (Shawbrook, WestOne). No formal TS yet.</t>
+          <t>Indic. 05/08: £5.6m, 70% LTV, 11%, 18m. Prideview SPV via Mantra. Borrower wants 24m.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="12.75" customHeight="1" s="105">
       <c r="A35" s="155" t="n">
-        <v>46235</v>
+        <v>46239</v>
       </c>
       <c r="B35" s="108" t="inlineStr">
         <is>
@@ -2805,27 +2805,27 @@
       </c>
       <c r="R35" s="108" t="inlineStr">
         <is>
-          <t>TS SIGNED + £15k commitment fee paid (early Sep). Net revised to £10.017m (was £9.72m) after borrower (Yoav) query; gross £10.8m, 11% fixed, 9mo, 1.75% arr fee, £243k exit; sized at 80% PP (£13.5m), broker cites min MV £17m. City Financial Mortgages / Manish Babla. Target completion early Sept - progressing to legals. Note: deal also out to multiple brokers / family offices.</t>
+          <t>TS signed + £15k commitment fee paid; net £10.02m, 11%, 9m. City Financial Mortgages. -&gt; legals, ~early-Sept completion.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="12.75" customHeight="1" s="105">
       <c r="A36" s="155" t="n">
-        <v>46235</v>
+        <v>46241</v>
       </c>
       <c r="B36" s="108" t="inlineStr">
         <is>
-          <t>London Retail Parade Portfolio (5 parades, 29 units - Woodford/E17/SE13/SE12/Bexley)</t>
+          <t>Flats 1 &amp; 2, De Vere Gardens, Kensington, W8</t>
         </is>
       </c>
       <c r="C36" s="120" t="inlineStr">
         <is>
-          <t>Mixed-use</t>
+          <t>Resi</t>
         </is>
       </c>
       <c r="D36" s="108" t="inlineStr">
         <is>
-          <t>Eastway Estates Ltd (Prideview Group)</t>
+          <t>Ladi (via IPCA Group)</t>
         </is>
       </c>
       <c r="E36" s="120" t="inlineStr">
@@ -2843,28 +2843,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H36" s="121" t="n">
-        <v>5.54</v>
-      </c>
-      <c r="I36" s="122" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="J36" s="121" t="n">
-        <v>5.6</v>
-      </c>
+      <c r="H36" s="121" t="n"/>
+      <c r="I36" s="122" t="n"/>
+      <c r="J36" s="121" t="n"/>
       <c r="K36" s="121" t="n">
-        <v>8</v>
-      </c>
-      <c r="L36" s="123">
-        <f>J36/K36</f>
-        <v/>
-      </c>
+        <v>4.5</v>
+      </c>
+      <c r="L36" s="123" t="n"/>
       <c r="M36" s="120" t="n">
-        <v>18</v>
-      </c>
-      <c r="N36" s="124" t="n">
-        <v>0.127</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="N36" s="124" t="n"/>
       <c r="O36" s="125" t="inlineStr">
         <is>
           <t>N</t>
@@ -2882,27 +2871,27 @@
       </c>
       <c r="R36" s="108" t="inlineStr">
         <is>
-          <t>Indicative terms 05/08 via Rickesh Patel (Mantra Commercial). Acquisition of 5 mixed-use retail parades (29 units) by Prideview SPV Eastway Estates Ltd. £5.6m at lower of 70% LTV (block value £8.0m) / 85.5% LTPP (PP £6.55m), 11% p.a., 1% arr, 1.5% exit, 18mo, PG 20%. Borrower requesting 24mo term / +6mo extension option. Value-add then refi/sell exit. No formal TS yet.</t>
+          <t>Enquiry 07/08: acq from receivers £4.5m. IPCA/Jignesh Desai. Terms TBC.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="105">
       <c r="A37" s="155" t="n">
-        <v>46235</v>
+        <v>46244</v>
       </c>
       <c r="B37" s="108" t="inlineStr">
         <is>
-          <t>Flats 1 &amp; 2, De Vere Gardens, Kensington, W8</t>
+          <t>Quadrant Shopping Centre, Dunstable, LU5 4RH</t>
         </is>
       </c>
       <c r="C37" s="120" t="inlineStr">
         <is>
-          <t>Resi</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="D37" s="108" t="inlineStr">
         <is>
-          <t>Ladi (via IPCA Group)</t>
+          <t>MGI Dunstable Ltd (Malhotra/Jain)</t>
         </is>
       </c>
       <c r="E37" s="120" t="inlineStr">
@@ -2920,17 +2909,28 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H37" s="121" t="n"/>
-      <c r="I37" s="122" t="n"/>
-      <c r="J37" s="121" t="n"/>
+      <c r="H37" s="121" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="I37" s="122" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J37" s="121" t="n">
+        <v>6.82</v>
+      </c>
       <c r="K37" s="121" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L37" s="123" t="n"/>
+        <v>8.52</v>
+      </c>
+      <c r="L37" s="123">
+        <f>J34/K34</f>
+        <v/>
+      </c>
       <c r="M37" s="120" t="n">
         <v>12</v>
       </c>
-      <c r="N37" s="124" t="n"/>
+      <c r="N37" s="124" t="n">
+        <v>0.145</v>
+      </c>
       <c r="O37" s="125" t="inlineStr">
         <is>
           <t>N</t>
@@ -2948,17 +2948,17 @@
       </c>
       <c r="R37" s="108" t="inlineStr">
         <is>
-          <t>Enquiry 07/08 via Jignesh Desai (IPCA Group). Acquisition of combined Flats 1&amp;2, De Vere Gardens, Kensington W8 by "Ladi" from receivers at £4.5m (was £7m 2yrs ago); expected rent ~£4,300pw. Targeting end-Aug drawdown. REL indicated 60-70% LTV, 9.0-10.8% p.a., 1% arr, 1% exit, 12mo - awaiting pack, loan amount TBC, no formal terms issued.</t>
+          <t>Indic. 12/08: £6.82m, 80% LTV, 12%, 12m. Fast Forward Capital. Borrower pushing 15m/nil-exit.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="105">
       <c r="A38" s="155" t="n">
-        <v>46266</v>
+        <v>46251</v>
       </c>
       <c r="B38" s="108" t="inlineStr">
         <is>
-          <t>SAL Hotels Limited (operating hotel)</t>
+          <t>St Giles Hotel, London</t>
         </is>
       </c>
       <c r="C38" s="120" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="D38" s="108" t="inlineStr">
         <is>
-          <t>SAL Hotels Ltd (via Mantra)</t>
+          <t>via Bridgemore Capital (Joe Eden)</t>
         </is>
       </c>
       <c r="E38" s="120" t="inlineStr">
@@ -2983,30 +2983,18 @@
       </c>
       <c r="G38" s="120" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H38" s="121" t="n">
-        <v>13.13</v>
-      </c>
-      <c r="I38" s="122" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="J38" s="121" t="n">
-        <v>13.5</v>
-      </c>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H38" s="121" t="n"/>
+      <c r="I38" s="122" t="n"/>
+      <c r="J38" s="121" t="n"/>
       <c r="K38" s="121" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="L38" s="123" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="M38" s="120" t="n">
-        <v>18</v>
-      </c>
-      <c r="N38" s="124" t="n">
-        <v>0.113</v>
-      </c>
+        <v>31.5</v>
+      </c>
+      <c r="L38" s="123" t="n"/>
+      <c r="M38" s="120" t="n"/>
+      <c r="N38" s="124" t="n"/>
       <c r="O38" s="125" t="inlineStr">
         <is>
           <t>N</t>
@@ -3024,27 +3012,27 @@
       </c>
       <c r="R38" s="108" t="inlineStr">
         <is>
-          <t>Active negotiation (Sep). REL terms 03/09: £13.5m (60% LTV / 79% of 180-day VPV), 10.5%, 1.25% REL arr fee + 1.5% Mantra fee, net Day-1 £13.13m. Refi/exit of Hilco debt; contract to Nov. Competing bid £14m/18mo at £140k arr. Mantra: Nirav Patel / Nimesh Sanghrajka. LTV/return indicative.</t>
+          <t>Enquiry 17/08: £31.5m hotel acq, IV ~£55m. Bridgemore. Terms TBC.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="12.75" customHeight="1" s="105">
       <c r="A39" s="155" t="n">
-        <v>46266</v>
+        <v>46251</v>
       </c>
       <c r="B39" s="108" t="inlineStr">
         <is>
-          <t>Resi Bridge - Aquilae (London resi, MV £11.5m)</t>
+          <t>Land loan - York (confidential)</t>
         </is>
       </c>
       <c r="C39" s="120" t="inlineStr">
         <is>
-          <t>Resi</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="D39" s="108" t="inlineStr">
         <is>
-          <t>via Aquilae Capital (Matthew Yassin)</t>
+          <t>via GLPG (Nick Swerner)</t>
         </is>
       </c>
       <c r="E39" s="120" t="inlineStr">
@@ -3062,30 +3050,16 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H39" s="121" t="n">
-        <v>6.53</v>
-      </c>
-      <c r="I39" s="122" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="J39" s="121" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="K39" s="121" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="L39" s="123" t="n">
-        <v>0.6435</v>
-      </c>
-      <c r="M39" s="120" t="n">
-        <v>12</v>
-      </c>
-      <c r="N39" s="124" t="n">
-        <v>0.117</v>
-      </c>
+      <c r="H39" s="121" t="n"/>
+      <c r="I39" s="122" t="n"/>
+      <c r="J39" s="121" t="n"/>
+      <c r="K39" s="121" t="n"/>
+      <c r="L39" s="123" t="n"/>
+      <c r="M39" s="120" t="n"/>
+      <c r="N39" s="124" t="n"/>
       <c r="O39" s="125" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P39" s="120" t="inlineStr">
@@ -3100,27 +3074,27 @@
       </c>
       <c r="R39" s="108" t="inlineStr">
         <is>
-          <t>Terms issued 04/09: £7.4m (65% LTV, MV £11.5m), 10.75%, 1% arr, £795k interest reserve (12m). Aquilae Capital / Matthew Yassin. Property address TBC.</t>
+          <t>Confidential land enquiry 17/08. GLPG/Nick Swerner. Details TBC.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="13.5" customHeight="1" s="105">
       <c r="A40" s="155" t="n">
-        <v>46235</v>
+        <v>46253</v>
       </c>
       <c r="B40" s="108" t="inlineStr">
         <is>
-          <t>Centre Heights, Swiss Cottage, NW3</t>
+          <t>Housing First Group / Serco portfolio (45 units/190 beds)</t>
         </is>
       </c>
       <c r="C40" s="120" t="inlineStr">
         <is>
-          <t>Mixed-use</t>
+          <t>Supported Living</t>
         </is>
       </c>
       <c r="D40" s="108" t="inlineStr">
         <is>
-          <t>via RIB (Adam Jaffe)</t>
+          <t>HFG (via GLPG - Nick Swerner)</t>
         </is>
       </c>
       <c r="E40" s="120" t="inlineStr">
@@ -3135,33 +3109,21 @@
       </c>
       <c r="G40" s="120" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H40" s="121" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="I40" s="122" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="J40" s="121" t="n">
-        <v>10.88</v>
-      </c>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H40" s="121" t="n"/>
+      <c r="I40" s="122" t="n"/>
+      <c r="J40" s="121" t="n"/>
       <c r="K40" s="121" t="n">
-        <v>16</v>
-      </c>
-      <c r="L40" s="123" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="M40" s="120" t="n">
-        <v>24</v>
-      </c>
-      <c r="N40" s="124" t="n">
-        <v>0.104</v>
-      </c>
+        <v>11.34</v>
+      </c>
+      <c r="L40" s="123" t="n"/>
+      <c r="M40" s="120" t="n"/>
+      <c r="N40" s="124" t="n"/>
       <c r="O40" s="125" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P40" s="120" t="inlineStr">
@@ -3176,27 +3138,27 @@
       </c>
       <c r="R40" s="108" t="inlineStr">
         <is>
-          <t>High-level terms 26/08: £10.88m (68% LTV), £272k interest reserve; 24-month term at 10.35% (35bps uplift for 24m vs 18m). REL keen ('very fundable'); full TS to be issued. RIB / Adam Jaffe. Return/net indicative.</t>
+          <t>TS in progress: 45 units/190 beds, MV £11.34m, Serco leases; GBB-funded. GLPG. Terms TBC.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="13.5" customHeight="1" s="105">
       <c r="A41" s="155" t="n">
-        <v>46235</v>
+        <v>46254</v>
       </c>
       <c r="B41" s="108" t="inlineStr">
         <is>
-          <t>Thorpe End (land / planning play)</t>
+          <t>26 Catherine Place, SW1E</t>
         </is>
       </c>
       <c r="C41" s="120" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Resi</t>
         </is>
       </c>
       <c r="D41" s="108" t="inlineStr">
         <is>
-          <t>via LS Capital (Jason Green)</t>
+          <t>via Opes (Masood Rashid)</t>
         </is>
       </c>
       <c r="E41" s="120" t="inlineStr">
@@ -3211,33 +3173,21 @@
       </c>
       <c r="G41" s="120" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H41" s="121" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="I41" s="122" t="n">
-        <v>0.23</v>
-      </c>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H41" s="121" t="n"/>
+      <c r="I41" s="122" t="n"/>
       <c r="J41" s="121" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="K41" s="121" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="L41" s="123" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M41" s="120" t="n">
-        <v>12</v>
-      </c>
-      <c r="N41" s="124" t="n">
-        <v>0.13</v>
-      </c>
+        <v>6.5</v>
+      </c>
+      <c r="K41" s="121" t="n"/>
+      <c r="L41" s="123" t="n"/>
+      <c r="M41" s="120" t="n"/>
+      <c r="N41" s="124" t="n"/>
       <c r="O41" s="125" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="P41" s="120" t="inlineStr">
@@ -3252,27 +3202,27 @@
       </c>
       <c r="R41" s="108" t="inlineStr">
         <is>
-          <t>Terms issued 28/08: gross £1.75m (50% LTV, MV land £3.5m / 70% of Saffron price), £210k interest reserve (12m, implies ~12%). Borrower interested, asked for pricing improvement (REL declined). Sale contract requested for underwrite. LS Capital / Jason Green.</t>
+          <t>Enquiry 20/08: £6.5m refinance. Opes/Masood Rashid. Terms TBC.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="155" t="n">
-        <v>46235</v>
+        <v>46255</v>
       </c>
       <c r="B42" s="108" t="inlineStr">
         <is>
-          <t>Housing First Group / Serco portfolio (45 units/190 beds)</t>
+          <t>Cranley Hotel</t>
         </is>
       </c>
       <c r="C42" s="120" t="inlineStr">
         <is>
-          <t>Supported Living</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D42" s="108" t="inlineStr">
         <is>
-          <t>HFG (via GLPG - Nick Swerner)</t>
+          <t>via BIZL (Pratik Shah)</t>
         </is>
       </c>
       <c r="E42" s="120" t="inlineStr">
@@ -3282,7 +3232,7 @@
       </c>
       <c r="F42" s="120" t="inlineStr">
         <is>
-          <t>Bridge</t>
+          <t>Term</t>
         </is>
       </c>
       <c r="G42" s="120" t="inlineStr">
@@ -3293,9 +3243,7 @@
       <c r="H42" s="121" t="n"/>
       <c r="I42" s="122" t="n"/>
       <c r="J42" s="121" t="n"/>
-      <c r="K42" s="121" t="n">
-        <v>11.34</v>
-      </c>
+      <c r="K42" s="121" t="n"/>
       <c r="L42" s="123" t="n"/>
       <c r="M42" s="120" t="n"/>
       <c r="N42" s="124" t="n"/>
@@ -3316,27 +3264,27 @@
       </c>
       <c r="R42" s="108" t="inlineStr">
         <is>
-          <t>TS in progress (Aug-Sep). Portfolio 45 units / 190 beds; MV (Serco leases) £11.34m, VPV (HMO) £11.5m; 6+6 leases. GBB funding appetite confirmed. Margin negotiation (~25bps gap). Loan amount/terms TBC. GLPG / Nick Swerner.</t>
+          <t>Enquiry 21/08: hotel refurb-to-term, bespoke structure. BIZL. Figures TBC.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="12.75" customHeight="1" s="105">
       <c r="A43" s="155" t="n">
-        <v>46235</v>
+        <v>46260</v>
       </c>
       <c r="B43" s="108" t="inlineStr">
         <is>
-          <t>St Giles Hotel, London</t>
+          <t>Centre Heights, Swiss Cottage, NW3</t>
         </is>
       </c>
       <c r="C43" s="120" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Mixed-use</t>
         </is>
       </c>
       <c r="D43" s="108" t="inlineStr">
         <is>
-          <t>via Bridgemore Capital (Joe Eden)</t>
+          <t>via RIB (Adam Jaffe)</t>
         </is>
       </c>
       <c r="E43" s="120" t="inlineStr">
@@ -3354,18 +3302,30 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H43" s="121" t="n"/>
-      <c r="I43" s="122" t="n"/>
-      <c r="J43" s="121" t="n"/>
+      <c r="H43" s="121" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="I43" s="122" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="J43" s="121" t="n">
+        <v>10.88</v>
+      </c>
       <c r="K43" s="121" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="L43" s="123" t="n"/>
-      <c r="M43" s="120" t="n"/>
-      <c r="N43" s="124" t="n"/>
+        <v>16</v>
+      </c>
+      <c r="L43" s="123" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="M43" s="120" t="n">
+        <v>24</v>
+      </c>
+      <c r="N43" s="124" t="n">
+        <v>0.104</v>
+      </c>
       <c r="O43" s="125" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P43" s="120" t="inlineStr">
@@ -3380,27 +3340,27 @@
       </c>
       <c r="R43" s="108" t="inlineStr">
         <is>
-          <t>Enquiry 17/08: £31.5m acquisition, investment value ~£55m. REL would size on lower of PP or MV. Loan amount/terms TBC. Bridgemore Capital / Joe Eden.</t>
+          <t>Terms 26/08: £10.88m, 68% LTV, 24m @10.35%. RIB/Adam Jaffe. Full TS to follow.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="13.8" customHeight="1" s="105">
       <c r="A44" s="155" t="n">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="B44" s="108" t="inlineStr">
         <is>
-          <t>Project Hannah - land bridge, London</t>
+          <t>Thorpe End (land / planning play)</t>
         </is>
       </c>
       <c r="C44" s="120" t="inlineStr">
         <is>
-          <t>Resi</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="D44" s="108" t="inlineStr">
         <is>
-          <t>via BLCK Capital (Delvin Kennedy)</t>
+          <t>via LS Capital (Jason Green)</t>
         </is>
       </c>
       <c r="E44" s="120" t="inlineStr">
@@ -3418,16 +3378,30 @@
           <t>A</t>
         </is>
       </c>
-      <c r="H44" s="121" t="n"/>
-      <c r="I44" s="122" t="n"/>
-      <c r="J44" s="121" t="n"/>
-      <c r="K44" s="121" t="n"/>
-      <c r="L44" s="123" t="n"/>
-      <c r="M44" s="120" t="n"/>
-      <c r="N44" s="124" t="n"/>
+      <c r="H44" s="121" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="I44" s="122" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="J44" s="121" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="K44" s="121" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L44" s="123" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M44" s="120" t="n">
+        <v>12</v>
+      </c>
+      <c r="N44" s="124" t="n">
+        <v>0.13</v>
+      </c>
       <c r="O44" s="125" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P44" s="120" t="inlineStr">
@@ -3442,7 +3416,7 @@
       </c>
       <c r="R44" s="108" t="inlineStr">
         <is>
-          <t>~£33m residential land bridge. NDA executed 07/09; info pack + memo + model received. Similar to Avanton Richmond scheme reviewed before. Given size, REL would partner with a preferred senior lender (loan-on-loan) - REL portion/terms TBC. BLCK Capital / Delvin Kennedy &amp; Jonathan Black.</t>
+          <t>Terms 28/08: £1.75m, 50% LTV, ~12%, 12m (land). LS Capital/Jason Green. Negotiating price.</t>
         </is>
       </c>
     </row>
@@ -3452,17 +3426,17 @@
       </c>
       <c r="B45" s="108" t="inlineStr">
         <is>
-          <t>Brighton Pier</t>
+          <t>SAL Hotels Limited (operating hotel)</t>
         </is>
       </c>
       <c r="C45" s="120" t="inlineStr">
         <is>
-          <t>Leisure</t>
+          <t>Hotel</t>
         </is>
       </c>
       <c r="D45" s="108" t="inlineStr">
         <is>
-          <t>via Yellowstone Finance (Dave Dixon)</t>
+          <t>SAL Hotels Ltd (via Mantra)</t>
         </is>
       </c>
       <c r="E45" s="120" t="inlineStr">
@@ -3477,18 +3451,30 @@
       </c>
       <c r="G45" s="120" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H45" s="121" t="n"/>
-      <c r="I45" s="122" t="n"/>
-      <c r="J45" s="121" t="n"/>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H45" s="121" t="n">
+        <v>13.13</v>
+      </c>
+      <c r="I45" s="122" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J45" s="121" t="n">
+        <v>13.5</v>
+      </c>
       <c r="K45" s="121" t="n">
-        <v>7</v>
-      </c>
-      <c r="L45" s="123" t="n"/>
-      <c r="M45" s="120" t="n"/>
-      <c r="N45" s="124" t="n"/>
+        <v>22.5</v>
+      </c>
+      <c r="L45" s="123" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="M45" s="120" t="n">
+        <v>18</v>
+      </c>
+      <c r="N45" s="124" t="n">
+        <v>0.113</v>
+      </c>
       <c r="O45" s="125" t="inlineStr">
         <is>
           <t>N</t>
@@ -3506,17 +3492,17 @@
       </c>
       <c r="R45" s="108" t="inlineStr">
         <is>
-          <t>Enquiry 07/09: £7m purchase. REL has seen it before (another bidder); would size against purchase price. Awaiting further details. Yellowstone Finance / Dave Dixon.</t>
+          <t>Neg. 03/09: £13.5m, 60% LTV, 10.5%, 18m; refi of Hilco. Mantra. Competing bid £14m.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="155" t="n">
-        <v>46235</v>
+        <v>46268</v>
       </c>
       <c r="B46" s="108" t="inlineStr">
         <is>
-          <t>26 Catherine Place, SW1E</t>
+          <t>Resi Bridge - Aquilae (London resi, MV £11.5m)</t>
         </is>
       </c>
       <c r="C46" s="120" t="inlineStr">
@@ -3526,7 +3512,7 @@
       </c>
       <c r="D46" s="108" t="inlineStr">
         <is>
-          <t>via Opes (Masood Rashid)</t>
+          <t>via Aquilae Capital (Matthew Yassin)</t>
         </is>
       </c>
       <c r="E46" s="120" t="inlineStr">
@@ -3541,21 +3527,33 @@
       </c>
       <c r="G46" s="120" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H46" s="121" t="n"/>
-      <c r="I46" s="122" t="n"/>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H46" s="121" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="I46" s="122" t="n">
+        <v>0.87</v>
+      </c>
       <c r="J46" s="121" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K46" s="121" t="n"/>
-      <c r="L46" s="123" t="n"/>
-      <c r="M46" s="120" t="n"/>
-      <c r="N46" s="124" t="n"/>
+        <v>7.4</v>
+      </c>
+      <c r="K46" s="121" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="L46" s="123" t="n">
+        <v>0.6435</v>
+      </c>
+      <c r="M46" s="120" t="n">
+        <v>12</v>
+      </c>
+      <c r="N46" s="124" t="n">
+        <v>0.117</v>
+      </c>
       <c r="O46" s="125" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="P46" s="120" t="inlineStr">
@@ -3570,37 +3568,37 @@
       </c>
       <c r="R46" s="108" t="inlineStr">
         <is>
-          <t>New bridging enquiry 20/08: £6.5m refinance. Terms not yet issued; value/LTV TBC. Opes / Masood Rashid.</t>
+          <t>Terms 04/09: £7.4m, 65% LTV, 10.75%, £795k IR, 12m. Aquilae/M. Yassin.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="155" t="n">
-        <v>46235</v>
+        <v>46268</v>
       </c>
       <c r="B47" s="108" t="inlineStr">
         <is>
-          <t>Cranley Hotel</t>
+          <t>DSH Southampton &amp; Whitsand Bay Fort Holiday Village</t>
         </is>
       </c>
       <c r="C47" s="120" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Leisure</t>
         </is>
       </c>
       <c r="D47" s="108" t="inlineStr">
         <is>
-          <t>via BIZL (Pratik Shah)</t>
+          <t>via Gemdar (Ramiah)</t>
         </is>
       </c>
       <c r="E47" s="120" t="inlineStr">
         <is>
-          <t>Senior</t>
+          <t>Mezz / 2nd charge</t>
         </is>
       </c>
       <c r="F47" s="120" t="inlineStr">
         <is>
-          <t>Term</t>
+          <t>Bridge</t>
         </is>
       </c>
       <c r="G47" s="120" t="inlineStr">
@@ -3610,7 +3608,9 @@
       </c>
       <c r="H47" s="121" t="n"/>
       <c r="I47" s="122" t="n"/>
-      <c r="J47" s="121" t="n"/>
+      <c r="J47" s="121" t="n">
+        <v>5</v>
+      </c>
       <c r="K47" s="121" t="n"/>
       <c r="L47" s="123" t="n"/>
       <c r="M47" s="120" t="n"/>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="R47" s="108" t="inlineStr">
         <is>
-          <t>Refurb-to-term. Bespoke structure proposed 27/08 (reduced initial interest burden) - figures TBC pending borrower response. REL previously looked at funding this hotel. BIZL / Pratik Shah.</t>
+          <t>Enquiry 03/09: client wants £5m 2nd charge; REL prefers wholeloan. Gemdar. Mismatch.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="155" t="n">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="B48" s="108" t="inlineStr">
         <is>
-          <t>DSH Southampton &amp; Whitsand Bay Fort Holiday Village</t>
+          <t>Project Hannah - land bridge, London</t>
         </is>
       </c>
       <c r="C48" s="120" t="inlineStr">
         <is>
-          <t>Leisure</t>
+          <t>Resi</t>
         </is>
       </c>
       <c r="D48" s="108" t="inlineStr">
         <is>
-          <t>via Gemdar (Ramiah)</t>
+          <t>via BLCK Capital (Delvin Kennedy)</t>
         </is>
       </c>
       <c r="E48" s="120" t="inlineStr">
         <is>
-          <t>Mezz / 2nd charge</t>
+          <t>Senior</t>
         </is>
       </c>
       <c r="F48" s="120" t="inlineStr">
@@ -3667,14 +3667,12 @@
       </c>
       <c r="G48" s="120" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H48" s="121" t="n"/>
       <c r="I48" s="122" t="n"/>
-      <c r="J48" s="121" t="n">
-        <v>5</v>
-      </c>
+      <c r="J48" s="121" t="n"/>
       <c r="K48" s="121" t="n"/>
       <c r="L48" s="123" t="n"/>
       <c r="M48" s="120" t="n"/>
@@ -3696,27 +3694,27 @@
       </c>
       <c r="R48" s="108" t="inlineStr">
         <is>
-          <t>Enquiry 03/09: client wants a £5m SECOND CHARGE. REL prefers a wholeloan (higher leverage across DSH Southampton + Whitsand Bay Fort Holiday Village). Structure mismatch - may not proceed unless client accepts wholeloan. Gemdar / Ramiah.</t>
+          <t>NDA 07/09: ~£33m resi land bridge. BLCK. REL to co-lend w/ senior - REL share TBC.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="155" t="n">
-        <v>46235</v>
+        <v>46272</v>
       </c>
       <c r="B49" s="108" t="inlineStr">
         <is>
-          <t>Land loan - York (confidential)</t>
+          <t>Brighton Pier</t>
         </is>
       </c>
       <c r="C49" s="120" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Leisure</t>
         </is>
       </c>
       <c r="D49" s="108" t="inlineStr">
         <is>
-          <t>via GLPG (Nick Swerner)</t>
+          <t>via Yellowstone Finance (Dave Dixon)</t>
         </is>
       </c>
       <c r="E49" s="120" t="inlineStr">
@@ -3737,7 +3735,9 @@
       <c r="H49" s="121" t="n"/>
       <c r="I49" s="122" t="n"/>
       <c r="J49" s="121" t="n"/>
-      <c r="K49" s="121" t="n"/>
+      <c r="K49" s="121" t="n">
+        <v>7</v>
+      </c>
       <c r="L49" s="123" t="n"/>
       <c r="M49" s="120" t="n"/>
       <c r="N49" s="124" t="n"/>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="R49" s="108" t="inlineStr">
         <is>
-          <t>Confidential land loan enquiry 17/08. Details/terms TBC. GLPG / Nick Swerner.</t>
+          <t>Enquiry 07/09: £7m purchase. Yellowstone/Dave Dixon. Awaiting details. (Poss. relates to Brighton Palace Pier row - confirm.)</t>
         </is>
       </c>
     </row>

</xml_diff>